<commit_message>
add an excel file
</commit_message>
<xml_diff>
--- a/Excel/green bond model.xlsx
+++ b/Excel/green bond model.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/066e823e8b38533c/Desktop/Green Bond ciments du maroc/Excel/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/066e823e8b38533c/Desktop/Green Bond ciments du maroc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8CFFAC37-FD88-4A18-8DB6-E8C3244A83A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8BD1BD96-190D-4FCB-888A-DF0A761A1C35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="2" activeTab="5" xr2:uid="{33557B9B-4A49-47B1-BABF-A87A4044C98D}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="10455" windowHeight="10905" firstSheet="3" activeTab="3" xr2:uid="{33557B9B-4A49-47B1-BABF-A87A4044C98D}"/>
   </bookViews>
   <sheets>
     <sheet name="00-COVER" sheetId="6" r:id="rId1"/>
@@ -179,6 +179,31 @@
     <author>Utilisateur</author>
   </authors>
   <commentList>
+    <comment ref="F7" authorId="0" shapeId="0" xr:uid="{716A58B6-8FC9-4A32-AC8D-0007A1B27E5E}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Utilisateur:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+sortie dargent 
+</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="M12" authorId="0" shapeId="0" xr:uid="{755037D0-3343-4552-846A-EBBAB4E816A9}">
       <text>
         <r>
@@ -352,7 +377,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="117">
   <si>
     <t>CA
 (operationnel)</t>
@@ -827,6 +852,13 @@
   <si>
     <t xml:space="preserve">Calcul de la VAN et le TRI :  </t>
   </si>
+  <si>
+    <t>Service de la
+ dette</t>
+  </si>
+  <si>
+    <t>DSCR</t>
+  </si>
 </sst>
 </file>
 
@@ -836,7 +868,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="30" x14ac:knownFonts="1">
+  <fonts count="31" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1051,6 +1083,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF787800"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -1142,7 +1181,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1200,15 +1239,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1248,9 +1278,6 @@
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1281,6 +1308,25 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="25" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1290,23 +1336,22 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="25" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1702,7 +1747,7 @@
       </c>
     </row>
     <row r="17" spans="13:31" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="M17" s="56" t="s">
+      <c r="M17" s="49" t="s">
         <v>107</v>
       </c>
       <c r="N17" s="1"/>
@@ -1746,7 +1791,7 @@
       <c r="AE18" s="1"/>
     </row>
     <row r="19" spans="13:31" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="M19" s="56" t="s">
+      <c r="M19" s="49" t="s">
         <v>108</v>
       </c>
       <c r="N19" s="1"/>
@@ -1790,7 +1835,7 @@
       <c r="AE20" s="1"/>
     </row>
     <row r="21" spans="13:31" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="M21" s="56" t="s">
+      <c r="M21" s="49" t="s">
         <v>109</v>
       </c>
       <c r="N21" s="1"/>
@@ -1831,26 +1876,26 @@
   <sheetData>
     <row r="5" spans="5:9" ht="29.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="6" spans="5:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E6" s="57" t="s">
+      <c r="E6" s="50" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="7" spans="5:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G7" s="31" t="s">
+      <c r="G7" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="31" t="s">
+      <c r="H7" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="I7" s="31" t="s">
+      <c r="I7" s="28" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="8" spans="5:9" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G8" s="29" t="s">
+      <c r="G8" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="24" t="s">
+      <c r="H8" s="21" t="s">
         <v>17</v>
       </c>
       <c r="I8" s="5" t="s">
@@ -1858,10 +1903,10 @@
       </c>
     </row>
     <row r="9" spans="5:9" ht="75" x14ac:dyDescent="0.25">
-      <c r="G9" s="29" t="s">
+      <c r="G9" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="H9" s="24" t="s">
+      <c r="H9" s="21" t="s">
         <v>18</v>
       </c>
       <c r="I9" s="5" t="s">
@@ -1869,10 +1914,10 @@
       </c>
     </row>
     <row r="10" spans="5:9" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G10" s="28" t="s">
+      <c r="G10" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="H10" s="24">
+      <c r="H10" s="21">
         <v>119</v>
       </c>
       <c r="I10" s="10" t="s">
@@ -1880,10 +1925,10 @@
       </c>
     </row>
     <row r="11" spans="5:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="G11" s="28" t="s">
+      <c r="G11" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="H11" s="24" t="s">
+      <c r="H11" s="21" t="s">
         <v>26</v>
       </c>
       <c r="I11" s="5" t="s">
@@ -1891,10 +1936,10 @@
       </c>
     </row>
     <row r="12" spans="5:9" ht="99.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G12" s="29" t="s">
+      <c r="G12" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="H12" s="24" t="s">
+      <c r="H12" s="21" t="s">
         <v>25</v>
       </c>
       <c r="I12" s="5" t="s">
@@ -1902,10 +1947,10 @@
       </c>
     </row>
     <row r="13" spans="5:9" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G13" s="29" t="s">
+      <c r="G13" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="H13" s="24" t="s">
+      <c r="H13" s="21" t="s">
         <v>31</v>
       </c>
       <c r="I13" s="5" t="s">
@@ -1913,10 +1958,10 @@
       </c>
     </row>
     <row r="14" spans="5:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G14" s="29" t="s">
+      <c r="G14" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="H14" s="24">
+      <c r="H14" s="21">
         <v>23.1</v>
       </c>
       <c r="I14" s="9" t="s">
@@ -1924,10 +1969,10 @@
       </c>
     </row>
     <row r="15" spans="5:9" ht="102.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G15" s="30" t="s">
+      <c r="G15" s="27" t="s">
         <v>34</v>
       </c>
-      <c r="H15" s="25">
+      <c r="H15" s="22">
         <v>0.04</v>
       </c>
       <c r="I15" s="17" t="s">
@@ -1935,10 +1980,10 @@
       </c>
     </row>
     <row r="16" spans="5:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="G16" s="30" t="s">
+      <c r="G16" s="27" t="s">
         <v>93</v>
       </c>
-      <c r="H16" s="25">
+      <c r="H16" s="22">
         <v>0.35</v>
       </c>
       <c r="I16" s="5" t="s">
@@ -1946,10 +1991,10 @@
       </c>
     </row>
     <row r="17" spans="7:9" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G17" s="30" t="s">
+      <c r="G17" s="27" t="s">
         <v>95</v>
       </c>
-      <c r="H17" s="25">
+      <c r="H17" s="22">
         <v>2.5999999999999999E-2</v>
       </c>
       <c r="I17" s="2" t="s">
@@ -1957,10 +2002,10 @@
       </c>
     </row>
     <row r="18" spans="7:9" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G18" s="29" t="s">
+      <c r="G18" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="H18" s="26">
+      <c r="H18" s="23">
         <v>0.08</v>
       </c>
       <c r="I18" s="5" t="s">
@@ -1968,10 +2013,10 @@
       </c>
     </row>
     <row r="19" spans="7:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="G19" s="29" t="s">
+      <c r="G19" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="H19" s="24">
+      <c r="H19" s="21">
         <v>1.8</v>
       </c>
       <c r="I19" s="5" t="s">
@@ -1979,10 +2024,10 @@
       </c>
     </row>
     <row r="20" spans="7:9" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G20" s="29" t="s">
+      <c r="G20" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="H20" s="24" t="s">
+      <c r="H20" s="21" t="s">
         <v>86</v>
       </c>
       <c r="I20" s="5" t="s">
@@ -1990,10 +2035,10 @@
       </c>
     </row>
     <row r="21" spans="7:9" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G21" s="29" t="s">
+      <c r="G21" s="26" t="s">
         <v>87</v>
       </c>
-      <c r="H21" s="24" t="s">
+      <c r="H21" s="21" t="s">
         <v>88</v>
       </c>
       <c r="I21" s="5" t="s">
@@ -2025,12 +2070,12 @@
       <c r="E4" s="1"/>
     </row>
     <row r="6" spans="2:8" ht="24" x14ac:dyDescent="0.4">
-      <c r="B6" s="58" t="s">
+      <c r="B6" s="51" t="s">
         <v>111</v>
       </c>
-      <c r="C6" s="58"/>
-      <c r="D6" s="58"/>
-      <c r="E6" s="58"/>
+      <c r="C6" s="51"/>
+      <c r="D6" s="51"/>
+      <c r="E6" s="51"/>
     </row>
     <row r="8" spans="2:8" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F8" s="7">
@@ -2044,7 +2089,7 @@
       </c>
     </row>
     <row r="9" spans="2:8" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E9" s="32" t="s">
+      <c r="E9" s="29" t="s">
         <v>0</v>
       </c>
       <c r="F9" s="6">
@@ -2058,7 +2103,7 @@
       </c>
     </row>
     <row r="10" spans="2:8" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E10" s="32" t="s">
+      <c r="E10" s="29" t="s">
         <v>1</v>
       </c>
       <c r="F10" s="6">
@@ -2072,7 +2117,7 @@
       </c>
     </row>
     <row r="11" spans="2:8" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="E11" s="32" t="s">
+      <c r="E11" s="29" t="s">
         <v>2</v>
       </c>
       <c r="F11" s="6">
@@ -2086,7 +2131,7 @@
       </c>
     </row>
     <row r="12" spans="2:8" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="E12" s="32" t="s">
+      <c r="E12" s="29" t="s">
         <v>3</v>
       </c>
       <c r="F12" s="6">
@@ -2114,7 +2159,7 @@
       </c>
     </row>
     <row r="14" spans="2:8" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E14" s="32" t="s">
+      <c r="E14" s="29" t="s">
         <v>5</v>
       </c>
       <c r="F14" s="6">
@@ -2128,7 +2173,7 @@
       </c>
     </row>
     <row r="15" spans="2:8" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E15" s="32" t="s">
+      <c r="E15" s="29" t="s">
         <v>91</v>
       </c>
       <c r="F15" s="20">
@@ -2170,24 +2215,24 @@
       </c>
     </row>
     <row r="18" spans="2:9" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E18" s="27" t="s">
+      <c r="E18" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="F18" s="33">
+      <c r="F18" s="30">
         <v>3193.4</v>
       </c>
-      <c r="G18" s="34">
+      <c r="G18" s="31">
         <v>3308.9</v>
       </c>
-      <c r="H18" s="34">
+      <c r="H18" s="31">
         <v>3197.8</v>
       </c>
     </row>
     <row r="19" spans="2:9" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E19" s="27" t="s">
+      <c r="E19" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="F19" s="35"/>
+      <c r="F19" s="32"/>
       <c r="G19" s="6">
         <v>166.2</v>
       </c>
@@ -2240,14 +2285,14 @@
       </c>
     </row>
     <row r="28" spans="2:9" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="D28" s="36" t="s">
+      <c r="D28" s="33" t="s">
         <v>101</v>
       </c>
-      <c r="F28" s="21" t="s">
+      <c r="F28" s="56" t="s">
         <v>112</v>
       </c>
-      <c r="G28" s="21"/>
-      <c r="H28" s="21"/>
+      <c r="G28" s="56"/>
+      <c r="H28" s="56"/>
       <c r="I28" s="14">
         <f>(H9-F9)/H9</f>
         <v>7.3556370302474791E-2</v>
@@ -2270,9 +2315,9 @@
       </c>
     </row>
     <row r="34" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E34" s="22"/>
-      <c r="F34" s="22"/>
-      <c r="G34" s="22"/>
+      <c r="E34" s="57"/>
+      <c r="F34" s="57"/>
+      <c r="G34" s="57"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2287,7 +2332,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9255B5B8-0016-4F10-BD3B-EBF84EC2F5C4}">
-  <dimension ref="D2:M13"/>
+  <dimension ref="D2:M15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="16.42578125" customWidth="1"/>
@@ -2296,35 +2341,35 @@
   <sheetData>
     <row r="2" spans="4:13" ht="24" x14ac:dyDescent="0.25">
       <c r="D2" s="1"/>
-      <c r="E2" s="59" t="s">
+      <c r="E2" s="52" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="3" spans="4:13" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G3" s="37" t="s">
+      <c r="G3" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="H3" s="37" t="s">
+      <c r="H3" s="34" t="s">
         <v>69</v>
       </c>
-      <c r="I3" s="37" t="s">
+      <c r="I3" s="34" t="s">
         <v>70</v>
       </c>
-      <c r="J3" s="37" t="s">
+      <c r="J3" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="K3" s="37" t="s">
+      <c r="K3" s="34" t="s">
         <v>72</v>
       </c>
-      <c r="L3" s="37" t="s">
+      <c r="L3" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="M3" s="37" t="s">
+      <c r="M3" s="34" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="4" spans="4:13" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F4" s="39" t="s">
+      <c r="F4" s="35" t="s">
         <v>40</v>
       </c>
       <c r="G4" s="8">
@@ -2357,7 +2402,7 @@
       </c>
     </row>
     <row r="5" spans="4:13" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F5" s="39" t="s">
+      <c r="F5" s="35" t="s">
         <v>41</v>
       </c>
       <c r="G5" s="8">
@@ -2390,7 +2435,7 @@
       </c>
     </row>
     <row r="6" spans="4:13" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="F6" s="39" t="s">
+      <c r="F6" s="35" t="s">
         <v>42</v>
       </c>
       <c r="G6" s="8">
@@ -2423,7 +2468,7 @@
       </c>
     </row>
     <row r="7" spans="4:13" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="F7" s="39" t="s">
+      <c r="F7" s="35" t="s">
         <v>43</v>
       </c>
       <c r="G7" s="8">
@@ -2456,7 +2501,7 @@
       </c>
     </row>
     <row r="8" spans="4:13" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="F8" s="39" t="s">
+      <c r="F8" s="35" t="s">
         <v>97</v>
       </c>
       <c r="G8" s="8">
@@ -2489,7 +2534,7 @@
       </c>
     </row>
     <row r="9" spans="4:13" ht="56.25" x14ac:dyDescent="0.3">
-      <c r="F9" s="40" t="s">
+      <c r="F9" s="36" t="s">
         <v>44</v>
       </c>
       <c r="G9" s="8">
@@ -2522,7 +2567,7 @@
       </c>
     </row>
     <row r="10" spans="4:13" ht="75" x14ac:dyDescent="0.3">
-      <c r="F10" s="40" t="s">
+      <c r="F10" s="36" t="s">
         <v>98</v>
       </c>
       <c r="G10" s="8">
@@ -2555,7 +2600,7 @@
       </c>
     </row>
     <row r="11" spans="4:13" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F11" s="39" t="s">
+      <c r="F11" s="35" t="s">
         <v>45</v>
       </c>
       <c r="G11" s="8">
@@ -2582,7 +2627,7 @@
       </c>
     </row>
     <row r="12" spans="4:13" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F12" s="41" t="s">
+      <c r="F12" s="37" t="s">
         <v>75</v>
       </c>
       <c r="G12" s="8">
@@ -2614,21 +2659,87 @@
         <v>127.44200000000001</v>
       </c>
     </row>
-    <row r="13" spans="4:13" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="F13" s="38" t="s">
+    <row r="13" spans="4:13" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F13" s="60" t="s">
+        <v>115</v>
+      </c>
+      <c r="G13" s="8">
+        <f>-(G7+G11)</f>
+        <v>4.76</v>
+      </c>
+      <c r="H13" s="8">
+        <f t="shared" ref="H13:M13" si="4">-(H7+H11)</f>
+        <v>4.76</v>
+      </c>
+      <c r="I13" s="8">
+        <f t="shared" si="4"/>
+        <v>4.76</v>
+      </c>
+      <c r="J13" s="8">
+        <f t="shared" si="4"/>
+        <v>4.76</v>
+      </c>
+      <c r="K13" s="8">
+        <f t="shared" si="4"/>
+        <v>4.76</v>
+      </c>
+      <c r="L13" s="8">
+        <f t="shared" si="4"/>
+        <v>4.76</v>
+      </c>
+      <c r="M13" s="8">
+        <f t="shared" si="4"/>
+        <v>123.76</v>
+      </c>
+    </row>
+    <row r="14" spans="4:13" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F14" s="61" t="s">
+        <v>116</v>
+      </c>
+      <c r="G14" s="8">
+        <f>G9/G13</f>
+        <v>3.4747899159663866</v>
+      </c>
+      <c r="H14" s="8">
+        <f t="shared" ref="H14:M14" si="5">H9/H13</f>
+        <v>3.4747899159663866</v>
+      </c>
+      <c r="I14" s="8">
+        <f t="shared" si="5"/>
+        <v>3.4747899159663866</v>
+      </c>
+      <c r="J14" s="8">
+        <f t="shared" si="5"/>
+        <v>3.4747899159663866</v>
+      </c>
+      <c r="K14" s="8">
+        <f t="shared" si="5"/>
+        <v>3.4747899159663866</v>
+      </c>
+      <c r="L14" s="8">
+        <f t="shared" si="5"/>
+        <v>3.4747899159663866</v>
+      </c>
+      <c r="M14" s="8">
+        <f t="shared" si="5"/>
+        <v>0.13364576599870717</v>
+      </c>
+    </row>
+    <row r="15" spans="4:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="F15" s="58" t="s">
         <v>67</v>
       </c>
-      <c r="G13" s="23"/>
-      <c r="H13" s="23"/>
-      <c r="I13" s="23"/>
-      <c r="J13" s="23"/>
-      <c r="K13" s="23"/>
-      <c r="L13" s="23"/>
-      <c r="M13" s="23"/>
+      <c r="G15" s="59"/>
+      <c r="H15" s="59"/>
+      <c r="I15" s="59"/>
+      <c r="J15" s="59"/>
+      <c r="K15" s="59"/>
+      <c r="L15" s="59"/>
+      <c r="M15" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="F13:M13"/>
+    <mergeCell ref="F15:M15"/>
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2654,7 +2765,7 @@
     <row r="3" spans="6:26" ht="31.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="6:26" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="6:26" ht="24.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="F5" s="46" t="s">
+      <c r="F5" s="42" t="s">
         <v>114</v>
       </c>
     </row>
@@ -2722,7 +2833,7 @@
       </c>
     </row>
     <row r="8" spans="6:26" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="F8" s="45" t="s">
+      <c r="F8" s="41" t="s">
         <v>46</v>
       </c>
       <c r="G8" s="8">
@@ -2896,26 +3007,26 @@
       <c r="G12" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="M12" s="43" t="s">
+      <c r="M12" s="39" t="s">
         <v>78</v>
       </c>
-      <c r="N12" s="43" t="s">
+      <c r="N12" s="39" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="13" spans="6:26" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F13" s="37" t="s">
+      <c r="F13" s="34" t="s">
         <v>77</v>
       </c>
       <c r="G13" s="8">
         <f>-'01-ASSUMPTIONS'!H10</f>
         <v>-119</v>
       </c>
-      <c r="M13" s="44">
+      <c r="M13" s="40">
         <f>NPV('01-ASSUMPTIONS'!$H$18,'04-VALUATION'!G8:Z8)+'04-VALUATION'!G13</f>
         <v>90.126539778669752</v>
       </c>
-      <c r="N13" s="42">
+      <c r="N13" s="38">
         <f>IRR(F9:Z9)</f>
         <v>0.17143215290529557</v>
       </c>
@@ -2947,94 +3058,94 @@
   </cols>
   <sheetData>
     <row r="5" spans="6:27" ht="26.25" x14ac:dyDescent="0.25">
-      <c r="H5" s="54" t="s">
+      <c r="H5" s="47" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="7" spans="6:27" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="J7" s="46"/>
-      <c r="K7" s="47" t="s">
+      <c r="J7" s="42"/>
+      <c r="K7" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="L7" s="48" t="s">
+      <c r="L7" s="44" t="s">
         <v>83</v>
       </c>
-      <c r="M7" s="53" t="s">
+      <c r="M7" s="46" t="s">
         <v>84</v>
       </c>
-      <c r="N7" s="48"/>
-      <c r="O7" s="48" t="s">
+      <c r="N7" s="44"/>
+      <c r="O7" s="44" t="s">
         <v>85</v>
       </c>
-      <c r="P7" s="48" t="s">
+      <c r="P7" s="44" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="8" spans="6:27" ht="26.25" x14ac:dyDescent="0.25">
-      <c r="J8" s="48" t="s">
+      <c r="J8" s="44" t="s">
         <v>80</v>
       </c>
-      <c r="K8" s="49">
+      <c r="K8" s="45">
         <v>1400</v>
       </c>
-      <c r="L8" s="49">
+      <c r="L8" s="45">
         <v>0.56000000000000005</v>
       </c>
-      <c r="M8" s="50">
+      <c r="M8" s="53">
         <v>15.3</v>
       </c>
-      <c r="N8" s="50"/>
-      <c r="O8" s="49">
+      <c r="N8" s="53"/>
+      <c r="O8" s="45">
         <f>-'01-ASSUMPTIONS'!$H$10+('05-SCENARIOS'!M8-'01-ASSUMPTIONS'!$H$19)*(1-(1+'01-ASSUMPTIONS'!$H$18)^-20)/'01-ASSUMPTIONS'!$H$18</f>
         <v>13.544990000565463</v>
       </c>
-      <c r="P8" s="55">
+      <c r="P8" s="48">
         <f>RATE(20,M8-'01-ASSUMPTIONS'!$H$19,-'01-ASSUMPTIONS'!$H$10)</f>
         <v>9.4960425220687095E-2</v>
       </c>
     </row>
     <row r="9" spans="6:27" ht="26.25" x14ac:dyDescent="0.25">
-      <c r="J9" s="48" t="s">
+      <c r="J9" s="44" t="s">
         <v>81</v>
       </c>
-      <c r="K9" s="49">
+      <c r="K9" s="45">
         <v>1700</v>
       </c>
-      <c r="L9" s="49">
+      <c r="L9" s="45">
         <v>0.8</v>
       </c>
-      <c r="M9" s="50">
+      <c r="M9" s="53">
         <v>23.1</v>
       </c>
-      <c r="N9" s="50"/>
-      <c r="O9" s="49">
+      <c r="N9" s="53"/>
+      <c r="O9" s="45">
         <f>-'01-ASSUMPTIONS'!$H$10+('05-SCENARIOS'!M9-'01-ASSUMPTIONS'!$H$19)*(1-(1+'01-ASSUMPTIONS'!$H$18)^-20)/'01-ASSUMPTIONS'!$H$18</f>
         <v>90.126539778669951</v>
       </c>
-      <c r="P9" s="55">
+      <c r="P9" s="48">
         <f>RATE(20,M9-'01-ASSUMPTIONS'!$H$19,-'01-ASSUMPTIONS'!$H$10)</f>
         <v>0.17143215290548311</v>
       </c>
     </row>
     <row r="10" spans="6:27" ht="26.25" x14ac:dyDescent="0.25">
-      <c r="J10" s="48" t="s">
+      <c r="J10" s="44" t="s">
         <v>82</v>
       </c>
-      <c r="K10" s="49">
+      <c r="K10" s="45">
         <v>1900</v>
       </c>
-      <c r="L10" s="49">
+      <c r="L10" s="45">
         <v>0.9</v>
       </c>
-      <c r="M10" s="51">
+      <c r="M10" s="54">
         <v>29.1</v>
       </c>
-      <c r="N10" s="52"/>
-      <c r="O10" s="49">
+      <c r="N10" s="55"/>
+      <c r="O10" s="45">
         <f>-'01-ASSUMPTIONS'!$H$10+('05-SCENARIOS'!M10-'01-ASSUMPTIONS'!$H$19)*(1-(1+'01-ASSUMPTIONS'!$H$18)^-20)/'01-ASSUMPTIONS'!$H$18</f>
         <v>149.03542422336568</v>
       </c>
-      <c r="P10" s="55">
+      <c r="P10" s="48">
         <f>IRR(F16:Z16)</f>
         <v>0.22548093237740363</v>
       </c>

</xml_diff>